<commit_message>
Si bien el codigo esta muy desordenado, es una primera iteracion que logra extraer datos de nuevos partidos y termina prediciendo un resultado.
Tiene el problema de que deduce el valor de variables muy importante para la prediccion que son las variables de jugadores (como dif_rat_tit, dif_edad_sup, dif_rat_aus) puesto que no pude extraer las formaciones
</commit_message>
<xml_diff>
--- a/data_preparation/data/etiquetas_equipo_ganador.xlsx
+++ b/data_preparation/data/etiquetas_equipo_ganador.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -470,6 +470,12 @@
         <v>2</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>